<commit_message>
docs(planning): update final-stretch plan and week schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/2026-10-06_week_schedule.xlsx
+++ b/documents/2026-10-06_week_schedule.xlsx
@@ -769,17 +769,17 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Pick the 2 clones: one per host, each comfortably above 50 ng/uL</t>
+          <t>SENT: 9-2-1 R1 and 9-6-2 R1</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>9-2-1 and 9-6-2 are the same strain by ANI (100.000%), so one clone from each gives guaranteed-independent lineages on a shared reference. R3 is the safer default - 9-2-1 R1 read only 55.8, too close to the 50 ng/uL floor</t>
+          <t>One clone per host. 9-2-1 and 9-6-2 are the same strain by ANI (100.000%), so one from each gives guaranteed-independent resistance events against a shared reference</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2 chosen clone IDs -&gt; planning doc</t>
+          <t>2 tubes shipped. R2/R3 x4 stay at 4 C fridge as the replication set</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -1004,17 +1004,17 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Streak the lawn panel from -80 C glycerol stocks: 9-2-1, 9-6-2, 3 non-host (+ 6 resistant if stocks exist)</t>
+          <t>Streak the 7-strain lawn panel from -80 C glycerol stocks</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Lawn panel for Thursday's spot test. Hosts and non-hosts are in the 28-stock panel; the resistant clones are the uncertain ones</t>
+          <t>hosts 9-2-1 + 9-6-2 (batch-1) | resistant 9-2-1 R1 + 9-6-2 R1 (July box, NOT in the 28-stock panel) | non-hosts 8-10-2 (batch-2), 10-10-2 (batch-1), 9-1-1 (batch-2)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>5-11 streak plates -&gt; 30 C incubator overnight</t>
+          <t>7 streak plates -&gt; 30 C incubator overnight. 5 plates if the resistant stocks are missing</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -3018,7 +3018,7 @@
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Which 3 non-host strains. 8-10-2 and 10-10-2 recommended: F for both phages on the 7/04 matrix and both have annotated genomes, so a halo can be tied straight to a sugar biosynthetic cassette.</t>
+          <t>Non-host panel settled: 8-10-2, 10-10-2, 9-1-1. All three are F for both phages on the 7/04 matrix. 8-10-2 and 10-10-2 have annotated genomes, so a halo ties straight to a sugar biosynthetic cassette; 8-10-2 is also a different species (P. capeferrum, ANI 98.66%). 9-1-1 is the same collection site as the hosts and its neighbour 9-1-2 is T/T positive, which makes it the cleanest near-pair contrast. Excluded: the site-6 group (the 7/14 contamination-or-prophage control was never read), 8-1-2 and 9-10-1 (ambiguity markers in the matrix), 8-5-1 (open label discrepancy with 8-3-1).</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
     <row r="38">
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Sequencing: 2 clones, one per host. 9-2-1 and 9-6-2 are the same strain by ANI (100.000%), so one from each gives guaranteed-independent resistance events against a shared reference. Choose after the re-Qubit, favouring R3 over R1 - 9-2-1 R1 read 55.8 ng/uL, too close to the 50 ng/uL floor. Keep the other four tubes as the replication set.</t>
+          <t>Sequencing: 9-2-1 R1 and 9-6-2 R1 sent. One clone per host, and since the two parents are the same strain by ANI (100.000%) these are guaranteed-independent resistance events against a shared reference. The same two clones are revived for the lawn panel, so halo phenotype and genome come from the same clone. R2/R3 x4 stay at 4 C as the replication set. Watch coverage on 9-2-1 R1 when the data lands - its July reading was the lowest of the six (55.8 ng/uL extrapolated).</t>
         </is>
       </c>
     </row>

</xml_diff>